<commit_message>
updated repo prior to manuscript submission
</commit_message>
<xml_diff>
--- a/Inputs/LEPA metrics.xlsx
+++ b/Inputs/LEPA metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gamtostyrimai-my.sharepoint.com/personal/nathan_baker_gamtc_lt/Documents/MOBILR Project (2024-2027)/Analyses/Operational taxalist/Calculating OTL indices/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{7F5854A3-E252-42E7-BA39-535C40055322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92202428-6209-4A9A-BBFA-80DBC5F6AFFE}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{7F5854A3-E252-42E7-BA39-535C40055322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A128A477-F4EB-4894-A146-700FB09B910C}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0B851701-A1B2-4D96-ADFF-67A0CCF28F8E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0B851701-A1B2-4D96-ADFF-67A0CCF28F8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Lapas1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="105">
   <si>
     <t>LTR1063</t>
   </si>
@@ -354,6 +354,9 @@
   </si>
   <si>
     <t>lepa_eqr_corrected</t>
+  </si>
+  <si>
+    <t>Bad</t>
   </si>
 </sst>
 </file>
@@ -746,25 +749,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F31B79-BB5D-4B69-B443-206AA39BE057}">
   <dimension ref="A1:M83"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.68359375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.3125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1015625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.47265625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.08984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.5234375" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.62890625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.26171875" customWidth="1"/>
+    <col min="11" max="11" width="6.54296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="28.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>91</v>
       </c>
@@ -805,7 +808,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -844,7 +847,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -883,7 +886,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -922,7 +925,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -961,7 +964,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1000,7 +1003,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1039,7 +1042,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1078,7 +1081,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1117,7 +1120,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1156,7 +1159,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1195,7 +1198,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1234,7 +1237,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1273,7 +1276,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1312,7 +1315,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1351,7 +1354,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1390,7 +1393,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1432,7 +1435,7 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1471,7 +1474,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1510,7 +1513,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1549,7 +1552,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1588,7 +1591,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1630,7 +1633,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1669,7 +1672,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1708,7 +1711,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1750,7 +1753,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1789,7 +1792,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1828,7 +1831,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1867,7 +1870,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1906,7 +1909,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1945,7 +1948,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1984,7 +1987,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -2023,7 +2026,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -2062,7 +2065,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -2101,7 +2104,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -2140,7 +2143,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -2179,7 +2182,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -2218,7 +2221,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -2260,7 +2263,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -2299,7 +2302,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -2338,7 +2341,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -2377,7 +2380,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -2416,7 +2419,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -2458,7 +2461,7 @@
         <v>0.71</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -2494,10 +2497,10 @@
         <v>0.23</v>
       </c>
       <c r="L44" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -2536,7 +2539,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -2575,7 +2578,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -2614,7 +2617,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -2653,7 +2656,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -2692,7 +2695,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -2731,7 +2734,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -2770,7 +2773,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -2809,7 +2812,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -2848,7 +2851,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -2887,7 +2890,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -2926,7 +2929,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -2965,7 +2968,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -3004,7 +3007,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -3043,7 +3046,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -3082,7 +3085,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -3121,7 +3124,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -3163,7 +3166,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -3202,7 +3205,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -3241,7 +3244,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -3280,7 +3283,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -3322,7 +3325,7 @@
         <v>0.73</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -3361,7 +3364,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -3400,7 +3403,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -3439,7 +3442,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -3478,7 +3481,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -3517,7 +3520,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -3556,7 +3559,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -3595,7 +3598,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -3634,7 +3637,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -3673,7 +3676,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -3712,7 +3715,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -3748,13 +3751,13 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="L76" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="M76">
         <v>0.25</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -3793,7 +3796,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -3832,7 +3835,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -3871,7 +3874,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -3910,7 +3913,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -3952,7 +3955,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -3991,7 +3994,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -4031,6 +4034,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M83" xr:uid="{C8F31B79-BB5D-4B69-B443-206AA39BE057}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>